<commit_message>
Deploying to gh-pages from @ yugandharreddy0718/smartstudyai@124040879bccbc2f72b4d26dea5adbe80c6e5c93 🚀
</commit_message>
<xml_diff>
--- a/reports/Mobile/appium-report.xlsx
+++ b/reports/Mobile/appium-report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="121">
   <si>
     <t>SMARTSTUDY AI - ANDROID APPIUM E2E TEST REPORT</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>18.59 seconds</t>
+    <t>18.61 seconds</t>
   </si>
   <si>
     <t>Execution Platform</t>
@@ -56,7 +56,7 @@
     <t>Date &amp; Time</t>
   </si>
   <si>
-    <t>8/21/2026, 1:31:59 PM</t>
+    <t>8/27/2026, 3:18:12 PM</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -98,10 +98,10 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:41.190Z</t>
-  </si>
-  <si>
-    <t>2026-08-21T13:31:42.392Z</t>
+    <t>2026-08-27T15:17:54.563Z</t>
+  </si>
+  <si>
+    <t>2026-08-27T15:17:55.764Z</t>
   </si>
   <si>
     <t>Verified successfully.</t>
@@ -116,7 +116,10 @@
     <t>Mobile Login Screen &amp; Form Rendering</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:42.993Z</t>
+    <t>2026-08-27T15:17:55.765Z</t>
+  </si>
+  <si>
+    <t>2026-08-27T15:17:56.366Z</t>
   </si>
   <si>
     <t>APP-003</t>
@@ -125,7 +128,7 @@
     <t>Invalid Mobile Login Error Handling</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:43.594Z</t>
+    <t>2026-08-27T15:17:56.967Z</t>
   </si>
   <si>
     <t>APP-004</t>
@@ -137,7 +140,7 @@
     <t>Student Dashboard &amp; Subject Grid Cards</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:44.195Z</t>
+    <t>2026-08-27T15:17:57.568Z</t>
   </si>
   <si>
     <t>APP-005</t>
@@ -149,7 +152,7 @@
     <t>Switch Active Grade to Class 6</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:44.796Z</t>
+    <t>2026-08-27T15:17:58.169Z</t>
   </si>
   <si>
     <t>APP-006</t>
@@ -158,7 +161,7 @@
     <t>Switch Active Grade to Class 7</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:45.397Z</t>
+    <t>2026-08-27T15:17:58.770Z</t>
   </si>
   <si>
     <t>APP-007</t>
@@ -167,7 +170,7 @@
     <t>Switch Active Grade to Class 8</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:45.998Z</t>
+    <t>2026-08-27T15:17:59.371Z</t>
   </si>
   <si>
     <t>APP-008</t>
@@ -176,7 +179,7 @@
     <t>Switch Active Grade to Class 9</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:46.599Z</t>
+    <t>2026-08-27T15:17:59.972Z</t>
   </si>
   <si>
     <t>APP-009</t>
@@ -185,7 +188,7 @@
     <t>Switch Active Grade to Class 10</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:47.201Z</t>
+    <t>2026-08-27T15:18:00.573Z</t>
   </si>
   <si>
     <t>APP-010</t>
@@ -197,7 +200,7 @@
     <t>Explore Mathematics Stream Grid</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:47.802Z</t>
+    <t>2026-08-27T15:18:01.174Z</t>
   </si>
   <si>
     <t>APP-011</t>
@@ -206,7 +209,7 @@
     <t>Explore Physics, Chemistry &amp; Biology Streams</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:48.403Z</t>
+    <t>2026-08-27T15:18:01.774Z</t>
   </si>
   <si>
     <t>APP-012</t>
@@ -215,7 +218,7 @@
     <t>Explore History, Civics &amp; Geography Streams</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:49.004Z</t>
+    <t>2026-08-27T15:18:02.376Z</t>
   </si>
   <si>
     <t>APP-013</t>
@@ -227,7 +230,7 @@
     <t>Chapter Catalog Navigation &amp; Sub-lesson Catalog</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:49.605Z</t>
+    <t>2026-08-27T15:18:02.977Z</t>
   </si>
   <si>
     <t>APP-014</t>
@@ -239,7 +242,7 @@
     <t>Verify 13-Section Pedagogical Layout Rendering</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:51.407Z</t>
+    <t>2026-08-27T15:18:04.780Z</t>
   </si>
   <si>
     <t>APP-015</t>
@@ -251,7 +254,7 @@
     <t>Trigger Mark Lesson Complete &amp; XP Award (+100 XP)</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:52.008Z</t>
+    <t>2026-08-27T15:18:05.381Z</t>
   </si>
   <si>
     <t>APP-016</t>
@@ -263,7 +266,7 @@
     <t>AI Studio — Interactive Summary Tool</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:52.609Z</t>
+    <t>2026-08-27T15:18:05.982Z</t>
   </si>
   <si>
     <t>APP-017</t>
@@ -275,7 +278,7 @@
     <t>AI Studio — High-Yield Exam Q&amp;A Generator</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:53.210Z</t>
+    <t>2026-08-27T15:18:06.583Z</t>
   </si>
   <si>
     <t>APP-018</t>
@@ -287,7 +290,7 @@
     <t>AI Studio — Standalone MCQ Generator</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:55.212Z</t>
+    <t>2026-08-27T15:18:08.585Z</t>
   </si>
   <si>
     <t>APP-019</t>
@@ -299,7 +302,7 @@
     <t>AI Studio — Interactive Quiz Assessment</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:55.813Z</t>
+    <t>2026-08-27T15:18:09.186Z</t>
   </si>
   <si>
     <t>APP-020</t>
@@ -311,7 +314,7 @@
     <t>AI Studio — 24/7 AI Tutor Chat Assistant Interface</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:56.414Z</t>
+    <t>2026-08-27T15:18:09.787Z</t>
   </si>
   <si>
     <t>APP-021</t>
@@ -323,7 +326,7 @@
     <t>Mobile Document Upload &amp; OCR Text Extraction Studio</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:57.015Z</t>
+    <t>2026-08-27T15:18:10.388Z</t>
   </si>
   <si>
     <t>APP-022</t>
@@ -335,7 +338,7 @@
     <t>Mobile PDF Reader &amp; Document Viewer Tools</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:57.616Z</t>
+    <t>2026-08-27T15:18:10.989Z</t>
   </si>
   <si>
     <t>APP-023</t>
@@ -347,7 +350,7 @@
     <t>Execute Search Query across Curriculum Index</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:58.217Z</t>
+    <t>2026-08-27T15:18:11.590Z</t>
   </si>
   <si>
     <t>APP-024</t>
@@ -359,7 +362,7 @@
     <t>Student Profile Stats &amp; Session Logout Execution</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:58.818Z</t>
+    <t>2026-08-27T15:18:12.191Z</t>
   </si>
   <si>
     <t>APP-025</t>
@@ -371,7 +374,7 @@
     <t>Protected Route Access Control &amp; Security Check</t>
   </si>
   <si>
-    <t>2026-08-21T13:31:59.419Z</t>
+    <t>2026-08-27T15:18:12.792Z</t>
   </si>
 </sst>
 </file>
@@ -946,7 +949,7 @@
         <v>27</v>
       </c>
       <c r="E2">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="F2" t="s">
         <v>28</v>
@@ -978,10 +981,10 @@
         <v>601</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H3" t="s">
         <v>30</v>
@@ -992,13 +995,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>27</v>
@@ -1007,10 +1010,10 @@
         <v>601</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H4" t="s">
         <v>30</v>
@@ -1021,25 +1024,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5">
+        <v>601</v>
+      </c>
+      <c r="F5" t="s">
         <v>38</v>
       </c>
-      <c r="B5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5">
-        <v>601</v>
-      </c>
-      <c r="F5" t="s">
-        <v>37</v>
-      </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
         <v>30</v>
@@ -1050,25 +1053,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6">
+        <v>601</v>
+      </c>
+      <c r="F6" t="s">
         <v>42</v>
       </c>
-      <c r="B6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6">
-        <v>601</v>
-      </c>
-      <c r="F6" t="s">
-        <v>41</v>
-      </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
         <v>30</v>
@@ -1079,25 +1082,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7">
+        <v>601</v>
+      </c>
+      <c r="F7" t="s">
         <v>46</v>
       </c>
-      <c r="B7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7">
-        <v>601</v>
-      </c>
-      <c r="F7" t="s">
-        <v>45</v>
-      </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H7" t="s">
         <v>30</v>
@@ -1108,25 +1111,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <v>601</v>
+      </c>
+      <c r="F8" t="s">
         <v>49</v>
       </c>
-      <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>601</v>
-      </c>
-      <c r="F8" t="s">
-        <v>48</v>
-      </c>
       <c r="G8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s">
         <v>30</v>
@@ -1137,25 +1140,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9">
+        <v>601</v>
+      </c>
+      <c r="F9" t="s">
         <v>52</v>
       </c>
-      <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9">
-        <v>601</v>
-      </c>
-      <c r="F9" t="s">
-        <v>51</v>
-      </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
         <v>30</v>
@@ -1166,25 +1169,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10">
+        <v>601</v>
+      </c>
+      <c r="F10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10">
-        <v>602</v>
-      </c>
-      <c r="F10" t="s">
-        <v>54</v>
-      </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H10" t="s">
         <v>30</v>
@@ -1195,25 +1198,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11">
+        <v>601</v>
+      </c>
+      <c r="F11" t="s">
         <v>58</v>
       </c>
-      <c r="B11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11">
-        <v>601</v>
-      </c>
-      <c r="F11" t="s">
-        <v>57</v>
-      </c>
       <c r="G11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H11" t="s">
         <v>30</v>
@@ -1224,25 +1227,25 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12">
+        <v>600</v>
+      </c>
+      <c r="F12" t="s">
         <v>62</v>
       </c>
-      <c r="B12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12">
-        <v>601</v>
-      </c>
-      <c r="F12" t="s">
-        <v>61</v>
-      </c>
       <c r="G12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H12" t="s">
         <v>30</v>
@@ -1253,25 +1256,25 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13">
+        <v>602</v>
+      </c>
+      <c r="F13" t="s">
         <v>65</v>
       </c>
-      <c r="B13" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13">
-        <v>601</v>
-      </c>
-      <c r="F13" t="s">
-        <v>64</v>
-      </c>
       <c r="G13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H13" t="s">
         <v>30</v>
@@ -1282,25 +1285,25 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14">
+        <v>601</v>
+      </c>
+      <c r="F14" t="s">
         <v>68</v>
       </c>
-      <c r="B14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" t="s">
-        <v>70</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14">
-        <v>601</v>
-      </c>
-      <c r="F14" t="s">
-        <v>67</v>
-      </c>
       <c r="G14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H14" t="s">
         <v>30</v>
@@ -1311,25 +1314,25 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15">
+        <v>1803</v>
+      </c>
+      <c r="F15" t="s">
         <v>72</v>
       </c>
-      <c r="B15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C15" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15">
-        <v>1802</v>
-      </c>
-      <c r="F15" t="s">
-        <v>71</v>
-      </c>
       <c r="G15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H15" t="s">
         <v>30</v>
@@ -1340,25 +1343,25 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16">
+        <v>601</v>
+      </c>
+      <c r="F16" t="s">
         <v>76</v>
       </c>
-      <c r="B16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C16" t="s">
-        <v>78</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16">
-        <v>601</v>
-      </c>
-      <c r="F16" t="s">
-        <v>75</v>
-      </c>
       <c r="G16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H16" t="s">
         <v>30</v>
@@ -1369,25 +1372,25 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17">
+        <v>601</v>
+      </c>
+      <c r="F17" t="s">
         <v>80</v>
       </c>
-      <c r="B17" t="s">
-        <v>81</v>
-      </c>
-      <c r="C17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17">
-        <v>601</v>
-      </c>
-      <c r="F17" t="s">
-        <v>79</v>
-      </c>
       <c r="G17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H17" t="s">
         <v>30</v>
@@ -1398,25 +1401,25 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18">
+        <v>601</v>
+      </c>
+      <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="B18" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" t="s">
-        <v>86</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18">
-        <v>601</v>
-      </c>
-      <c r="F18" t="s">
-        <v>83</v>
-      </c>
       <c r="G18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H18" t="s">
         <v>30</v>
@@ -1427,13 +1430,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>27</v>
@@ -1442,10 +1445,10 @@
         <v>2002</v>
       </c>
       <c r="F19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H19" t="s">
         <v>30</v>
@@ -1456,25 +1459,25 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" t="s">
+        <v>94</v>
+      </c>
+      <c r="C20" t="s">
+        <v>95</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20">
+        <v>601</v>
+      </c>
+      <c r="F20" t="s">
         <v>92</v>
       </c>
-      <c r="B20" t="s">
-        <v>93</v>
-      </c>
-      <c r="C20" t="s">
-        <v>94</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20">
-        <v>601</v>
-      </c>
-      <c r="F20" t="s">
-        <v>91</v>
-      </c>
       <c r="G20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H20" t="s">
         <v>30</v>
@@ -1485,25 +1488,25 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>97</v>
+      </c>
+      <c r="B21" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21">
+        <v>601</v>
+      </c>
+      <c r="F21" t="s">
         <v>96</v>
       </c>
-      <c r="B21" t="s">
-        <v>97</v>
-      </c>
-      <c r="C21" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21">
-        <v>601</v>
-      </c>
-      <c r="F21" t="s">
-        <v>95</v>
-      </c>
       <c r="G21" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H21" t="s">
         <v>30</v>
@@ -1514,25 +1517,25 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22">
+        <v>601</v>
+      </c>
+      <c r="F22" t="s">
         <v>100</v>
       </c>
-      <c r="B22" t="s">
-        <v>101</v>
-      </c>
-      <c r="C22" t="s">
-        <v>102</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E22">
-        <v>601</v>
-      </c>
-      <c r="F22" t="s">
-        <v>99</v>
-      </c>
       <c r="G22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H22" t="s">
         <v>30</v>
@@ -1543,25 +1546,25 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>105</v>
+      </c>
+      <c r="B23" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23">
+        <v>601</v>
+      </c>
+      <c r="F23" t="s">
         <v>104</v>
       </c>
-      <c r="B23" t="s">
-        <v>105</v>
-      </c>
-      <c r="C23" t="s">
-        <v>106</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23">
-        <v>601</v>
-      </c>
-      <c r="F23" t="s">
-        <v>103</v>
-      </c>
       <c r="G23" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H23" t="s">
         <v>30</v>
@@ -1572,25 +1575,25 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24">
+        <v>601</v>
+      </c>
+      <c r="F24" t="s">
         <v>108</v>
       </c>
-      <c r="B24" t="s">
-        <v>109</v>
-      </c>
-      <c r="C24" t="s">
-        <v>110</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24">
-        <v>601</v>
-      </c>
-      <c r="F24" t="s">
-        <v>107</v>
-      </c>
       <c r="G24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H24" t="s">
         <v>30</v>
@@ -1601,25 +1604,25 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25">
+        <v>601</v>
+      </c>
+      <c r="F25" t="s">
         <v>112</v>
       </c>
-      <c r="B25" t="s">
-        <v>113</v>
-      </c>
-      <c r="C25" t="s">
-        <v>114</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E25">
-        <v>601</v>
-      </c>
-      <c r="F25" t="s">
-        <v>111</v>
-      </c>
       <c r="G25" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H25" t="s">
         <v>30</v>
@@ -1630,25 +1633,25 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26">
+        <v>601</v>
+      </c>
+      <c r="F26" t="s">
         <v>116</v>
       </c>
-      <c r="B26" t="s">
-        <v>117</v>
-      </c>
-      <c r="C26" t="s">
-        <v>118</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26">
-        <v>601</v>
-      </c>
-      <c r="F26" t="s">
-        <v>115</v>
-      </c>
       <c r="G26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H26" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ yugandharreddy0718/smartstudyai@d0d275136eb63a236d7dd2adc768a7ecdcb29133 🚀
</commit_message>
<xml_diff>
--- a/reports/Mobile/appium-report.xlsx
+++ b/reports/Mobile/appium-report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="122">
   <si>
     <t>SMARTSTUDY AI - ANDROID APPIUM E2E TEST REPORT</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>18.61 seconds</t>
+    <t>18.59 seconds</t>
   </si>
   <si>
     <t>Execution Platform</t>
@@ -56,7 +56,7 @@
     <t>Date &amp; Time</t>
   </si>
   <si>
-    <t>8/27/2026, 3:19:43 PM</t>
+    <t>8/27/2026, 4:40:05 PM</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -98,10 +98,10 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:25.712Z</t>
-  </si>
-  <si>
-    <t>2026-08-27T15:19:26.914Z</t>
+    <t>2026-08-27T16:39:46.812Z</t>
+  </si>
+  <si>
+    <t>2026-08-27T16:39:48.014Z</t>
   </si>
   <si>
     <t>Verified successfully.</t>
@@ -116,7 +116,7 @@
     <t>Mobile Login Screen &amp; Form Rendering</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:27.515Z</t>
+    <t>2026-08-27T16:39:48.615Z</t>
   </si>
   <si>
     <t>APP-003</t>
@@ -125,7 +125,7 @@
     <t>Invalid Mobile Login Error Handling</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:28.116Z</t>
+    <t>2026-08-27T16:39:49.216Z</t>
   </si>
   <si>
     <t>APP-004</t>
@@ -137,7 +137,10 @@
     <t>Student Dashboard &amp; Subject Grid Cards</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:28.718Z</t>
+    <t>2026-08-27T16:39:49.217Z</t>
+  </si>
+  <si>
+    <t>2026-08-27T16:39:49.819Z</t>
   </si>
   <si>
     <t>APP-005</t>
@@ -149,7 +152,7 @@
     <t>Switch Active Grade to Class 6</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:29.319Z</t>
+    <t>2026-08-27T16:39:50.420Z</t>
   </si>
   <si>
     <t>APP-006</t>
@@ -158,7 +161,7 @@
     <t>Switch Active Grade to Class 7</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:29.920Z</t>
+    <t>2026-08-27T16:39:51.021Z</t>
   </si>
   <si>
     <t>APP-007</t>
@@ -167,7 +170,7 @@
     <t>Switch Active Grade to Class 8</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:30.521Z</t>
+    <t>2026-08-27T16:39:51.622Z</t>
   </si>
   <si>
     <t>APP-008</t>
@@ -176,7 +179,7 @@
     <t>Switch Active Grade to Class 9</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:31.122Z</t>
+    <t>2026-08-27T16:39:52.223Z</t>
   </si>
   <si>
     <t>APP-009</t>
@@ -185,7 +188,7 @@
     <t>Switch Active Grade to Class 10</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:31.723Z</t>
+    <t>2026-08-27T16:39:52.825Z</t>
   </si>
   <si>
     <t>APP-010</t>
@@ -197,7 +200,7 @@
     <t>Explore Mathematics Stream Grid</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:32.324Z</t>
+    <t>2026-08-27T16:39:53.425Z</t>
   </si>
   <si>
     <t>APP-011</t>
@@ -206,7 +209,10 @@
     <t>Explore Physics, Chemistry &amp; Biology Streams</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:32.924Z</t>
+    <t>2026-08-27T16:39:53.426Z</t>
+  </si>
+  <si>
+    <t>2026-08-27T16:39:54.026Z</t>
   </si>
   <si>
     <t>APP-012</t>
@@ -215,7 +221,7 @@
     <t>Explore History, Civics &amp; Geography Streams</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:33.525Z</t>
+    <t>2026-08-27T16:39:54.628Z</t>
   </si>
   <si>
     <t>APP-013</t>
@@ -227,7 +233,7 @@
     <t>Chapter Catalog Navigation &amp; Sub-lesson Catalog</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:34.126Z</t>
+    <t>2026-08-27T16:39:55.228Z</t>
   </si>
   <si>
     <t>APP-014</t>
@@ -239,7 +245,7 @@
     <t>Verify 13-Section Pedagogical Layout Rendering</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:35.928Z</t>
+    <t>2026-08-27T16:39:57.030Z</t>
   </si>
   <si>
     <t>APP-015</t>
@@ -251,7 +257,7 @@
     <t>Trigger Mark Lesson Complete &amp; XP Award (+100 XP)</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:36.529Z</t>
+    <t>2026-08-27T16:39:57.631Z</t>
   </si>
   <si>
     <t>APP-016</t>
@@ -263,7 +269,7 @@
     <t>AI Studio — Interactive Summary Tool</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:37.129Z</t>
+    <t>2026-08-27T16:39:58.233Z</t>
   </si>
   <si>
     <t>APP-017</t>
@@ -275,7 +281,7 @@
     <t>AI Studio — High-Yield Exam Q&amp;A Generator</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:37.730Z</t>
+    <t>2026-08-27T16:39:58.834Z</t>
   </si>
   <si>
     <t>APP-018</t>
@@ -287,7 +293,7 @@
     <t>AI Studio — Standalone MCQ Generator</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:39.733Z</t>
+    <t>2026-08-27T16:40:00.836Z</t>
   </si>
   <si>
     <t>APP-019</t>
@@ -299,7 +305,7 @@
     <t>AI Studio — Interactive Quiz Assessment</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:40.334Z</t>
+    <t>2026-08-27T16:40:01.437Z</t>
   </si>
   <si>
     <t>APP-020</t>
@@ -311,7 +317,7 @@
     <t>AI Studio — 24/7 AI Tutor Chat Assistant Interface</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:40.935Z</t>
+    <t>2026-08-27T16:40:02.038Z</t>
   </si>
   <si>
     <t>APP-021</t>
@@ -323,7 +329,7 @@
     <t>Mobile Document Upload &amp; OCR Text Extraction Studio</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:41.536Z</t>
+    <t>2026-08-27T16:40:02.639Z</t>
   </si>
   <si>
     <t>APP-022</t>
@@ -335,7 +341,7 @@
     <t>Mobile PDF Reader &amp; Document Viewer Tools</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:42.137Z</t>
+    <t>2026-08-27T16:40:03.240Z</t>
   </si>
   <si>
     <t>APP-023</t>
@@ -347,7 +353,7 @@
     <t>Execute Search Query across Curriculum Index</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:42.738Z</t>
+    <t>2026-08-27T16:40:03.841Z</t>
   </si>
   <si>
     <t>APP-024</t>
@@ -359,7 +365,7 @@
     <t>Student Profile Stats &amp; Session Logout Execution</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:43.339Z</t>
+    <t>2026-08-27T16:40:04.442Z</t>
   </si>
   <si>
     <t>APP-025</t>
@@ -371,7 +377,7 @@
     <t>Protected Route Access Control &amp; Security Check</t>
   </si>
   <si>
-    <t>2026-08-27T15:19:43.940Z</t>
+    <t>2026-08-27T16:40:05.043Z</t>
   </si>
 </sst>
 </file>
@@ -1036,10 +1042,10 @@
         <v>602</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
         <v>30</v>
@@ -1050,13 +1056,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>27</v>
@@ -1065,10 +1071,10 @@
         <v>601</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
         <v>30</v>
@@ -1079,13 +1085,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>27</v>
@@ -1094,10 +1100,10 @@
         <v>601</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H7" t="s">
         <v>30</v>
@@ -1108,13 +1114,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>27</v>
@@ -1123,10 +1129,10 @@
         <v>601</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s">
         <v>30</v>
@@ -1137,13 +1143,13 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>27</v>
@@ -1152,10 +1158,10 @@
         <v>601</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
         <v>30</v>
@@ -1166,25 +1172,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10">
+        <v>602</v>
+      </c>
+      <c r="F10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10">
-        <v>601</v>
-      </c>
-      <c r="F10" t="s">
-        <v>54</v>
-      </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H10" t="s">
         <v>30</v>
@@ -1195,13 +1201,13 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>27</v>
@@ -1210,10 +1216,10 @@
         <v>601</v>
       </c>
       <c r="F11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H11" t="s">
         <v>30</v>
@@ -1224,13 +1230,13 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>27</v>
@@ -1239,10 +1245,10 @@
         <v>600</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H12" t="s">
         <v>30</v>
@@ -1253,25 +1259,25 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13">
+        <v>602</v>
+      </c>
+      <c r="F13" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13">
-        <v>601</v>
-      </c>
-      <c r="F13" t="s">
-        <v>64</v>
-      </c>
       <c r="G13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
         <v>30</v>
@@ -1282,25 +1288,25 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14">
+        <v>600</v>
+      </c>
+      <c r="F14" t="s">
         <v>69</v>
       </c>
-      <c r="C14" t="s">
-        <v>70</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14">
-        <v>601</v>
-      </c>
-      <c r="F14" t="s">
-        <v>67</v>
-      </c>
       <c r="G14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H14" t="s">
         <v>30</v>
@@ -1311,13 +1317,13 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>27</v>
@@ -1326,10 +1332,10 @@
         <v>1802</v>
       </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H15" t="s">
         <v>30</v>
@@ -1340,13 +1346,13 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>27</v>
@@ -1355,10 +1361,10 @@
         <v>601</v>
       </c>
       <c r="F16" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H16" t="s">
         <v>30</v>
@@ -1369,25 +1375,25 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B17" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17">
+        <v>602</v>
+      </c>
+      <c r="F17" t="s">
         <v>81</v>
       </c>
-      <c r="C17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17">
-        <v>600</v>
-      </c>
-      <c r="F17" t="s">
-        <v>79</v>
-      </c>
       <c r="G17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H17" t="s">
         <v>30</v>
@@ -1398,13 +1404,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>27</v>
@@ -1413,10 +1419,10 @@
         <v>601</v>
       </c>
       <c r="F18" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H18" t="s">
         <v>30</v>
@@ -1427,25 +1433,25 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
+        <v>92</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19">
+        <v>2002</v>
+      </c>
+      <c r="F19" t="s">
         <v>89</v>
       </c>
-      <c r="C19" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19">
-        <v>2003</v>
-      </c>
-      <c r="F19" t="s">
-        <v>87</v>
-      </c>
       <c r="G19" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H19" t="s">
         <v>30</v>
@@ -1456,13 +1462,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>27</v>
@@ -1471,10 +1477,10 @@
         <v>601</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G20" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H20" t="s">
         <v>30</v>
@@ -1485,13 +1491,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>27</v>
@@ -1500,10 +1506,10 @@
         <v>601</v>
       </c>
       <c r="F21" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H21" t="s">
         <v>30</v>
@@ -1514,13 +1520,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>27</v>
@@ -1529,10 +1535,10 @@
         <v>601</v>
       </c>
       <c r="F22" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G22" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H22" t="s">
         <v>30</v>
@@ -1543,13 +1549,13 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C23" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>27</v>
@@ -1558,10 +1564,10 @@
         <v>601</v>
       </c>
       <c r="F23" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G23" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H23" t="s">
         <v>30</v>
@@ -1572,13 +1578,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>27</v>
@@ -1587,10 +1593,10 @@
         <v>601</v>
       </c>
       <c r="F24" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G24" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H24" t="s">
         <v>30</v>
@@ -1601,13 +1607,13 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C25" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>27</v>
@@ -1616,10 +1622,10 @@
         <v>601</v>
       </c>
       <c r="F25" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H25" t="s">
         <v>30</v>
@@ -1630,13 +1636,13 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>27</v>
@@ -1645,10 +1651,10 @@
         <v>601</v>
       </c>
       <c r="F26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G26" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H26" t="s">
         <v>30</v>

</xml_diff>